<commit_message>
Correction des erreurs qa bb1b48418d843cc97953720b9410281f36435bb1
</commit_message>
<xml_diff>
--- a/qaErrors/ig/StructureDefinition-fr-composition-document-ips.xlsx
+++ b/qaErrors/ig/StructureDefinition-fr-composition-document-ips.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20476" uniqueCount="1343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20476" uniqueCount="1344">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-24T11:21:48+00:00</t>
+    <t>2026-09-24T12:14:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3442,7 +3442,7 @@
     <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
   &lt;coding&gt;
     &lt;system value="http://loinc.org"/&gt;
-    &lt;code value="11369-9"/&gt;
+    &lt;code value="11369-6"/&gt;
   &lt;/coding&gt;
 &lt;/valueCodeableConcept&gt;</t>
   </si>
@@ -3873,6 +3873,10 @@
   </si>
   <si>
     <t>Composition.section:sectionPregnancyHistory.entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">profile:resolve()}
+</t>
   </si>
   <si>
     <t>Composition.section:sectionPregnancyHistory.entry:historiqueGrossesse</t>
@@ -60665,7 +60669,7 @@
         <v>78</v>
       </c>
       <c r="AB480" t="s" s="2">
-        <v>915</v>
+        <v>1225</v>
       </c>
       <c r="AC480" s="2"/>
       <c r="AD480" t="s" s="2">
@@ -60707,13 +60711,13 @@
     </row>
     <row r="481" hidden="true">
       <c r="A481" t="s" s="2">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="B481" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C481" t="s" s="2">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="D481" t="s" s="2">
         <v>78</v>
@@ -60735,10 +60739,10 @@
         <v>78</v>
       </c>
       <c r="K481" t="s" s="2">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="L481" t="s" s="2">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="M481" t="s" s="2">
         <v>876</v>
@@ -60826,13 +60830,13 @@
     </row>
     <row r="482" hidden="true">
       <c r="A482" t="s" s="2">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="B482" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C482" t="s" s="2">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="D482" t="s" s="2">
         <v>78</v>
@@ -60854,10 +60858,10 @@
         <v>78</v>
       </c>
       <c r="K482" t="s" s="2">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="L482" t="s" s="2">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="M482" t="s" s="2">
         <v>876</v>
@@ -60945,7 +60949,7 @@
     </row>
     <row r="483">
       <c r="A483" t="s" s="2">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="B483" t="s" s="2">
         <v>881</v>
@@ -61062,7 +61066,7 @@
     </row>
     <row r="484" hidden="true">
       <c r="A484" t="s" s="2">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="B484" t="s" s="2">
         <v>889</v>
@@ -61179,13 +61183,13 @@
     </row>
     <row r="485">
       <c r="A485" t="s" s="2">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B485" t="s" s="2">
         <v>812</v>
       </c>
       <c r="C485" t="s" s="2">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="D485" t="s" s="2">
         <v>78</v>
@@ -61210,10 +61214,10 @@
         <v>568</v>
       </c>
       <c r="L485" t="s" s="2">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="M485" t="s" s="2">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="N485" s="2"/>
       <c r="O485" s="2"/>
@@ -61296,7 +61300,7 @@
     </row>
     <row r="486" hidden="true">
       <c r="A486" t="s" s="2">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="B486" t="s" s="2">
         <v>820</v>
@@ -61411,7 +61415,7 @@
     </row>
     <row r="487" hidden="true">
       <c r="A487" t="s" s="2">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="B487" t="s" s="2">
         <v>821</v>
@@ -61524,7 +61528,7 @@
     </row>
     <row r="488" hidden="true">
       <c r="A488" t="s" s="2">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="B488" t="s" s="2">
         <v>821</v>
@@ -61641,7 +61645,7 @@
     </row>
     <row r="489" hidden="true">
       <c r="A489" t="s" s="2">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="B489" t="s" s="2">
         <v>821</v>
@@ -61760,7 +61764,7 @@
     </row>
     <row r="490" hidden="true">
       <c r="A490" t="s" s="2">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="B490" t="s" s="2">
         <v>830</v>
@@ -61879,7 +61883,7 @@
     </row>
     <row r="491">
       <c r="A491" t="s" s="2">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="B491" t="s" s="2">
         <v>831</v>
@@ -61908,7 +61912,7 @@
         <v>105</v>
       </c>
       <c r="L491" t="s" s="2">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="M491" t="s" s="2">
         <v>834</v>
@@ -61998,7 +62002,7 @@
     </row>
     <row r="492">
       <c r="A492" t="s" s="2">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="B492" t="s" s="2">
         <v>837</v>
@@ -62046,7 +62050,7 @@
         <v>78</v>
       </c>
       <c r="S492" t="s" s="2">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="T492" t="s" s="2">
         <v>78</v>
@@ -62115,7 +62119,7 @@
     </row>
     <row r="493" hidden="true">
       <c r="A493" t="s" s="2">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="B493" t="s" s="2">
         <v>843</v>
@@ -62232,7 +62236,7 @@
     </row>
     <row r="494" hidden="true">
       <c r="A494" t="s" s="2">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="B494" t="s" s="2">
         <v>847</v>
@@ -62349,7 +62353,7 @@
     </row>
     <row r="495">
       <c r="A495" t="s" s="2">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="B495" t="s" s="2">
         <v>852</v>
@@ -62378,7 +62382,7 @@
         <v>182</v>
       </c>
       <c r="L495" t="s" s="2">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="M495" t="s" s="2">
         <v>854</v>
@@ -62466,7 +62470,7 @@
     </row>
     <row r="496" hidden="true">
       <c r="A496" t="s" s="2">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="B496" t="s" s="2">
         <v>858</v>
@@ -62585,7 +62589,7 @@
     </row>
     <row r="497" hidden="true">
       <c r="A497" t="s" s="2">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B497" t="s" s="2">
         <v>866</v>
@@ -62704,7 +62708,7 @@
     </row>
     <row r="498" hidden="true">
       <c r="A498" t="s" s="2">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="B498" t="s" s="2">
         <v>874</v>
@@ -62819,13 +62823,13 @@
     </row>
     <row r="499" hidden="true">
       <c r="A499" t="s" s="2">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="B499" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C499" t="s" s="2">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="D499" t="s" s="2">
         <v>78</v>
@@ -62847,10 +62851,10 @@
         <v>78</v>
       </c>
       <c r="K499" t="s" s="2">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="L499" t="s" s="2">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="M499" t="s" s="2">
         <v>876</v>
@@ -62938,13 +62942,13 @@
     </row>
     <row r="500" hidden="true">
       <c r="A500" t="s" s="2">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="B500" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C500" t="s" s="2">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="D500" t="s" s="2">
         <v>78</v>
@@ -62966,10 +62970,10 @@
         <v>78</v>
       </c>
       <c r="K500" t="s" s="2">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="L500" t="s" s="2">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="M500" t="s" s="2">
         <v>876</v>
@@ -63057,13 +63061,13 @@
     </row>
     <row r="501" hidden="true">
       <c r="A501" t="s" s="2">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="B501" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C501" t="s" s="2">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="D501" t="s" s="2">
         <v>78</v>
@@ -63085,10 +63089,10 @@
         <v>78</v>
       </c>
       <c r="K501" t="s" s="2">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="L501" t="s" s="2">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="M501" t="s" s="2">
         <v>876</v>
@@ -63176,7 +63180,7 @@
     </row>
     <row r="502">
       <c r="A502" t="s" s="2">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="B502" t="s" s="2">
         <v>881</v>
@@ -63293,7 +63297,7 @@
     </row>
     <row r="503" hidden="true">
       <c r="A503" t="s" s="2">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="B503" t="s" s="2">
         <v>889</v>
@@ -63410,13 +63414,13 @@
     </row>
     <row r="504">
       <c r="A504" t="s" s="2">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="B504" t="s" s="2">
         <v>812</v>
       </c>
       <c r="C504" t="s" s="2">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="D504" t="s" s="2">
         <v>78</v>
@@ -63441,10 +63445,10 @@
         <v>568</v>
       </c>
       <c r="L504" t="s" s="2">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="M504" t="s" s="2">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="N504" s="2"/>
       <c r="O504" s="2"/>
@@ -63527,7 +63531,7 @@
     </row>
     <row r="505" hidden="true">
       <c r="A505" t="s" s="2">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="B505" t="s" s="2">
         <v>820</v>
@@ -63642,7 +63646,7 @@
     </row>
     <row r="506" hidden="true">
       <c r="A506" t="s" s="2">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="B506" t="s" s="2">
         <v>821</v>
@@ -63755,7 +63759,7 @@
     </row>
     <row r="507" hidden="true">
       <c r="A507" t="s" s="2">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="B507" t="s" s="2">
         <v>821</v>
@@ -63872,7 +63876,7 @@
     </row>
     <row r="508" hidden="true">
       <c r="A508" t="s" s="2">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="B508" t="s" s="2">
         <v>821</v>
@@ -63991,7 +63995,7 @@
     </row>
     <row r="509" hidden="true">
       <c r="A509" t="s" s="2">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="B509" t="s" s="2">
         <v>830</v>
@@ -64110,7 +64114,7 @@
     </row>
     <row r="510">
       <c r="A510" t="s" s="2">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="B510" t="s" s="2">
         <v>831</v>
@@ -64139,7 +64143,7 @@
         <v>105</v>
       </c>
       <c r="L510" t="s" s="2">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="M510" t="s" s="2">
         <v>834</v>
@@ -64229,7 +64233,7 @@
     </row>
     <row r="511">
       <c r="A511" t="s" s="2">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="B511" t="s" s="2">
         <v>837</v>
@@ -64277,7 +64281,7 @@
         <v>78</v>
       </c>
       <c r="S511" t="s" s="2">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="T511" t="s" s="2">
         <v>78</v>
@@ -64346,7 +64350,7 @@
     </row>
     <row r="512" hidden="true">
       <c r="A512" t="s" s="2">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="B512" t="s" s="2">
         <v>843</v>
@@ -64463,7 +64467,7 @@
     </row>
     <row r="513" hidden="true">
       <c r="A513" t="s" s="2">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="B513" t="s" s="2">
         <v>847</v>
@@ -64580,7 +64584,7 @@
     </row>
     <row r="514">
       <c r="A514" t="s" s="2">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="B514" t="s" s="2">
         <v>852</v>
@@ -64609,7 +64613,7 @@
         <v>182</v>
       </c>
       <c r="L514" t="s" s="2">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="M514" t="s" s="2">
         <v>854</v>
@@ -64697,7 +64701,7 @@
     </row>
     <row r="515" hidden="true">
       <c r="A515" t="s" s="2">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="B515" t="s" s="2">
         <v>858</v>
@@ -64816,7 +64820,7 @@
     </row>
     <row r="516" hidden="true">
       <c r="A516" t="s" s="2">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="B516" t="s" s="2">
         <v>866</v>
@@ -64935,7 +64939,7 @@
     </row>
     <row r="517" hidden="true">
       <c r="A517" t="s" s="2">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="B517" t="s" s="2">
         <v>874</v>
@@ -65050,13 +65054,13 @@
     </row>
     <row r="518" hidden="true">
       <c r="A518" t="s" s="2">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="B518" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C518" t="s" s="2">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="D518" t="s" s="2">
         <v>78</v>
@@ -65078,10 +65082,10 @@
         <v>78</v>
       </c>
       <c r="K518" t="s" s="2">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="L518" t="s" s="2">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="M518" t="s" s="2">
         <v>876</v>
@@ -65169,7 +65173,7 @@
     </row>
     <row r="519">
       <c r="A519" t="s" s="2">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="B519" t="s" s="2">
         <v>881</v>
@@ -65286,7 +65290,7 @@
     </row>
     <row r="520" hidden="true">
       <c r="A520" t="s" s="2">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="B520" t="s" s="2">
         <v>889</v>
@@ -65403,13 +65407,13 @@
     </row>
     <row r="521">
       <c r="A521" t="s" s="2">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="B521" t="s" s="2">
         <v>812</v>
       </c>
       <c r="C521" t="s" s="2">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="D521" t="s" s="2">
         <v>78</v>
@@ -65434,10 +65438,10 @@
         <v>568</v>
       </c>
       <c r="L521" t="s" s="2">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="M521" t="s" s="2">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="N521" s="2"/>
       <c r="O521" s="2"/>
@@ -65520,7 +65524,7 @@
     </row>
     <row r="522" hidden="true">
       <c r="A522" t="s" s="2">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="B522" t="s" s="2">
         <v>820</v>
@@ -65635,7 +65639,7 @@
     </row>
     <row r="523" hidden="true">
       <c r="A523" t="s" s="2">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="B523" t="s" s="2">
         <v>821</v>
@@ -65748,7 +65752,7 @@
     </row>
     <row r="524" hidden="true">
       <c r="A524" t="s" s="2">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="B524" t="s" s="2">
         <v>821</v>
@@ -65865,7 +65869,7 @@
     </row>
     <row r="525" hidden="true">
       <c r="A525" t="s" s="2">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="B525" t="s" s="2">
         <v>821</v>
@@ -65984,7 +65988,7 @@
     </row>
     <row r="526" hidden="true">
       <c r="A526" t="s" s="2">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="B526" t="s" s="2">
         <v>830</v>
@@ -66103,7 +66107,7 @@
     </row>
     <row r="527">
       <c r="A527" t="s" s="2">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="B527" t="s" s="2">
         <v>831</v>
@@ -66132,7 +66136,7 @@
         <v>105</v>
       </c>
       <c r="L527" t="s" s="2">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="M527" t="s" s="2">
         <v>834</v>
@@ -66222,7 +66226,7 @@
     </row>
     <row r="528">
       <c r="A528" t="s" s="2">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="B528" t="s" s="2">
         <v>837</v>
@@ -66270,7 +66274,7 @@
         <v>78</v>
       </c>
       <c r="S528" t="s" s="2">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="T528" t="s" s="2">
         <v>78</v>
@@ -66339,7 +66343,7 @@
     </row>
     <row r="529" hidden="true">
       <c r="A529" t="s" s="2">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="B529" t="s" s="2">
         <v>843</v>
@@ -66456,7 +66460,7 @@
     </row>
     <row r="530" hidden="true">
       <c r="A530" t="s" s="2">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="B530" t="s" s="2">
         <v>847</v>
@@ -66573,7 +66577,7 @@
     </row>
     <row r="531">
       <c r="A531" t="s" s="2">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B531" t="s" s="2">
         <v>852</v>
@@ -66602,7 +66606,7 @@
         <v>182</v>
       </c>
       <c r="L531" t="s" s="2">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="M531" t="s" s="2">
         <v>854</v>
@@ -66690,7 +66694,7 @@
     </row>
     <row r="532" hidden="true">
       <c r="A532" t="s" s="2">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="B532" t="s" s="2">
         <v>858</v>
@@ -66809,7 +66813,7 @@
     </row>
     <row r="533" hidden="true">
       <c r="A533" t="s" s="2">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="B533" t="s" s="2">
         <v>866</v>
@@ -66928,7 +66932,7 @@
     </row>
     <row r="534" hidden="true">
       <c r="A534" t="s" s="2">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="B534" t="s" s="2">
         <v>874</v>
@@ -67043,13 +67047,13 @@
     </row>
     <row r="535" hidden="true">
       <c r="A535" t="s" s="2">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="B535" t="s" s="2">
         <v>874</v>
       </c>
       <c r="C535" t="s" s="2">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="D535" t="s" s="2">
         <v>78</v>
@@ -67071,10 +67075,10 @@
         <v>78</v>
       </c>
       <c r="K535" t="s" s="2">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="L535" t="s" s="2">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="M535" t="s" s="2">
         <v>876</v>
@@ -67162,7 +67166,7 @@
     </row>
     <row r="536">
       <c r="A536" t="s" s="2">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="B536" t="s" s="2">
         <v>881</v>
@@ -67279,7 +67283,7 @@
     </row>
     <row r="537" hidden="true">
       <c r="A537" t="s" s="2">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="B537" t="s" s="2">
         <v>889</v>
@@ -67396,13 +67400,13 @@
     </row>
     <row r="538">
       <c r="A538" t="s" s="2">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="B538" t="s" s="2">
         <v>812</v>
       </c>
       <c r="C538" t="s" s="2">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="D538" t="s" s="2">
         <v>78</v>
@@ -67427,10 +67431,10 @@
         <v>568</v>
       </c>
       <c r="L538" t="s" s="2">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="M538" t="s" s="2">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="N538" s="2"/>
       <c r="O538" s="2"/>
@@ -67513,7 +67517,7 @@
     </row>
     <row r="539" hidden="true">
       <c r="A539" t="s" s="2">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="B539" t="s" s="2">
         <v>820</v>
@@ -67628,7 +67632,7 @@
     </row>
     <row r="540" hidden="true">
       <c r="A540" t="s" s="2">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="B540" t="s" s="2">
         <v>821</v>
@@ -67741,7 +67745,7 @@
     </row>
     <row r="541" hidden="true">
       <c r="A541" t="s" s="2">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="B541" t="s" s="2">
         <v>821</v>
@@ -67858,7 +67862,7 @@
     </row>
     <row r="542" hidden="true">
       <c r="A542" t="s" s="2">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="B542" t="s" s="2">
         <v>821</v>
@@ -67977,7 +67981,7 @@
     </row>
     <row r="543" hidden="true">
       <c r="A543" t="s" s="2">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="B543" t="s" s="2">
         <v>830</v>
@@ -68096,7 +68100,7 @@
     </row>
     <row r="544">
       <c r="A544" t="s" s="2">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="B544" t="s" s="2">
         <v>831</v>
@@ -68125,7 +68129,7 @@
         <v>105</v>
       </c>
       <c r="L544" t="s" s="2">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="M544" t="s" s="2">
         <v>834</v>
@@ -68215,7 +68219,7 @@
     </row>
     <row r="545">
       <c r="A545" t="s" s="2">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="B545" t="s" s="2">
         <v>837</v>
@@ -68263,7 +68267,7 @@
         <v>78</v>
       </c>
       <c r="S545" t="s" s="2">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="T545" t="s" s="2">
         <v>78</v>
@@ -68332,7 +68336,7 @@
     </row>
     <row r="546" hidden="true">
       <c r="A546" t="s" s="2">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B546" t="s" s="2">
         <v>843</v>
@@ -68449,7 +68453,7 @@
     </row>
     <row r="547" hidden="true">
       <c r="A547" t="s" s="2">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B547" t="s" s="2">
         <v>847</v>
@@ -68566,7 +68570,7 @@
     </row>
     <row r="548">
       <c r="A548" t="s" s="2">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="B548" t="s" s="2">
         <v>852</v>
@@ -68595,7 +68599,7 @@
         <v>182</v>
       </c>
       <c r="L548" t="s" s="2">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="M548" t="s" s="2">
         <v>854</v>
@@ -68683,7 +68687,7 @@
     </row>
     <row r="549" hidden="true">
       <c r="A549" t="s" s="2">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B549" t="s" s="2">
         <v>858</v>
@@ -68802,7 +68806,7 @@
     </row>
     <row r="550" hidden="true">
       <c r="A550" t="s" s="2">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="B550" t="s" s="2">
         <v>866</v>
@@ -68921,7 +68925,7 @@
     </row>
     <row r="551" hidden="true">
       <c r="A551" t="s" s="2">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B551" t="s" s="2">
         <v>874</v>
@@ -69038,7 +69042,7 @@
     </row>
     <row r="552" hidden="true">
       <c r="A552" t="s" s="2">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B552" t="s" s="2">
         <v>881</v>
@@ -69157,7 +69161,7 @@
     </row>
     <row r="553" hidden="true">
       <c r="A553" t="s" s="2">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="B553" t="s" s="2">
         <v>889</v>

</xml_diff>